<commit_message>
test: Añadimos predicciones cuando N = 16000 y N = 32000
</commit_message>
<xml_diff>
--- a/Resultados/Resultados.xlsx
+++ b/Resultados/Resultados.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>N</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>x2</t>
+  </si>
+  <si>
+    <t>PREDICCIONES</t>
   </si>
 </sst>
 </file>
@@ -44,7 +47,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -59,6 +62,11 @@
     </font>
     <font>
       <sz val="13.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -78,7 +86,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border/>
     <border>
       <left style="thin">
@@ -146,6 +154,30 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -154,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -189,6 +221,18 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="9" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="11" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -408,6 +452,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="17.0"/>
     <col customWidth="1" min="2" max="5" width="20.63"/>
   </cols>
   <sheetData>
@@ -495,6 +540,49 @@
         <v>7</v>
       </c>
     </row>
+    <row r="9" ht="32.25" customHeight="1">
+      <c r="A9" s="12"/>
+      <c r="B9" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" ht="32.25" customHeight="1">
+      <c r="B10" s="14">
+        <v>16000.0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1167.302</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0.215</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.034</v>
+      </c>
+    </row>
+    <row r="11" ht="32.25" customHeight="1">
+      <c r="B11" s="15">
+        <v>32000.0</v>
+      </c>
+      <c r="C11" s="8">
+        <v>9338.418</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0.86</v>
+      </c>
+      <c r="E11" s="10">
+        <v>0.068</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>